<commit_message>
refactor: implement consistent back navigation and UI layout updates across tender management modules
</commit_message>
<xml_diff>
--- a/src/pages/tender/tenders/view tenders/zero cost/Rate analysis/RANEW.xlsx
+++ b/src/pages/tender/tenders/view tenders/zero cost/Rate analysis/RANEW.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/techi/Romaa/ExcelTemp/Tender/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/techi/Romaa/Romaa_FE/src/pages/tender/tenders/view tenders/zero cost/Rate analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CF6443D-B6FC-2745-BB2B-74EDEC029681}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08C096A9-1824-F443-A2B4-64404FADFD9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{7A680C2C-A4BA-4FED-AA6B-5FB628350A41}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{7A680C2C-A4BA-4FED-AA6B-5FB628350A41}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="779" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="108">
   <si>
     <t>ABS001</t>
   </si>
@@ -340,6 +340,24 @@
   </si>
   <si>
     <t>Contract</t>
+  </si>
+  <si>
+    <t>Machinery</t>
+  </si>
+  <si>
+    <t>Fuel</t>
+  </si>
+  <si>
+    <t>Contractor</t>
+  </si>
+  <si>
+    <t>NMR</t>
+  </si>
+  <si>
+    <t>Bulk Material</t>
+  </si>
+  <si>
+    <t>Consumable</t>
   </si>
 </sst>
 </file>
@@ -765,7 +783,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{260209C6-4614-4F46-8222-CEC2192D5132}">
-  <dimension ref="A1:G202"/>
+  <dimension ref="A1:M202"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.33203125" style="2" customWidth="1"/>
@@ -776,7 +794,7 @@
     <col min="7" max="7" width="9.83203125" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
@@ -799,7 +817,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" s="9" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="10" t="s">
         <v>0</v>
       </c>
@@ -816,7 +834,7 @@
       </c>
       <c r="G2" s="10"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -839,7 +857,7 @@
         <v>6500</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>2</v>
       </c>
@@ -862,7 +880,7 @@
         <v>5384.62</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>3</v>
       </c>
@@ -884,8 +902,14 @@
       <c r="G5" s="2">
         <v>96</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="L5" t="s">
+        <v>3</v>
+      </c>
+      <c r="M5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>4</v>
       </c>
@@ -907,8 +931,14 @@
       <c r="G6" s="2">
         <v>700</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L6" t="s">
+        <v>6</v>
+      </c>
+      <c r="M6" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" s="9" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="10" t="s">
         <v>13</v>
       </c>
@@ -924,8 +954,14 @@
         <v>87.57</v>
       </c>
       <c r="G7" s="10"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="L7" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="M7" s="9" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>1</v>
       </c>
@@ -947,8 +983,14 @@
       <c r="G8" s="2">
         <v>5384.62</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="L8" t="s">
+        <v>10</v>
+      </c>
+      <c r="M8" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>2</v>
       </c>
@@ -970,8 +1012,14 @@
       <c r="G9" s="2">
         <v>96</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="L9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M9" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>3</v>
       </c>
@@ -993,8 +1041,14 @@
       <c r="G10" s="2">
         <v>700</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="L10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M10" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" s="9" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
         <v>27</v>
       </c>
@@ -1011,7 +1065,7 @@
       </c>
       <c r="G11" s="8"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>1</v>
       </c>
@@ -1034,7 +1088,7 @@
         <v>5384.62</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>2</v>
       </c>
@@ -1057,7 +1111,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>3</v>
       </c>
@@ -1080,7 +1134,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="15" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" s="9" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
         <v>28</v>
       </c>
@@ -1097,7 +1151,7 @@
       </c>
       <c r="G15" s="8"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>1</v>
       </c>

</xml_diff>